<commit_message>
📊 Actualizar CV_VU.xlsx — 24-03-2026, 11:11:44 a. m.
</commit_message>
<xml_diff>
--- a/datos/CV_VU.xlsx
+++ b/datos/CV_VU.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anais Gonzales\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{566A9B27-5412-4086-8423-E7C155DC65BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F34CD0B-5A3D-40ED-A98A-0207545A63D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -481,7 +481,7 @@
     <t>espinozabernardo1@gmail.com; ; ; ;</t>
   </si>
   <si>
-    <t>NICOLAS ROMERO</t>
+    <t>GABRIELA DEL CARMEN ROJAS QUEZADA</t>
   </si>
   <si>
     <t>Maria Clarisa Arraño Morales</t>
@@ -601,6 +601,9 @@
     <t>24 - Quilicura - Santiago -CP</t>
   </si>
   <si>
+    <t>949464419</t>
+  </si>
+  <si>
     <t>950009831</t>
   </si>
   <si>
@@ -791,9 +794,6 @@
   </si>
   <si>
     <t>alexandra.natalie.vs@gmail.com; ; ; ;</t>
-  </si>
-  <si>
-    <t>GABRIELA DEL CARMEN ROJAS QUEZADA</t>
   </si>
   <si>
     <t>Margarita Cristina Rojas Quezada</t>
@@ -1819,7 +1819,8 @@
   <dimension ref="A1:AP19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="42" width="8" customWidth="1"/>
+    <col min="1" max="41" width="8" customWidth="1"/>
+    <col min="42" max="42" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.3">
@@ -3000,13 +3001,13 @@
         <v>193</v>
       </c>
       <c r="I10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L10" t="s">
         <v>169</v>
@@ -3021,10 +3022,10 @@
         <v>87</v>
       </c>
       <c r="P10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Q10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R10" t="s">
         <v>90</v>
@@ -3048,19 +3049,19 @@
         <v>94</v>
       </c>
       <c r="Y10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Z10" t="s">
         <v>95</v>
       </c>
       <c r="AA10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AB10" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AC10" t="s">
-        <v>160</v>
+        <v>67</v>
       </c>
       <c r="AD10" t="s">
         <v>98</v>
@@ -3099,7 +3100,7 @@
         <v>49</v>
       </c>
       <c r="AP10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.3">
@@ -3110,28 +3111,28 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H11" t="s">
         <v>49</v>
       </c>
       <c r="I11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="J11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="K11" t="s">
         <v>156</v>
@@ -3152,16 +3153,16 @@
         <v>137</v>
       </c>
       <c r="Q11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="S11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="T11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="U11" t="s">
         <v>60</v>
@@ -3173,22 +3174,22 @@
         <v>93</v>
       </c>
       <c r="X11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Y11" t="s">
         <v>169</v>
       </c>
       <c r="Z11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="AA11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="AB11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AC11" t="s">
-        <v>160</v>
+        <v>67</v>
       </c>
       <c r="AD11" t="s">
         <v>68</v>
@@ -3227,7 +3228,7 @@
         <v>187</v>
       </c>
       <c r="AP11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.3">
@@ -3238,34 +3239,34 @@
         <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D12" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E12" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F12" t="s">
         <v>47</v>
       </c>
       <c r="G12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H12" t="s">
         <v>49</v>
       </c>
       <c r="I12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="L12" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="M12" t="s">
         <v>54</v>
@@ -3298,22 +3299,22 @@
         <v>60</v>
       </c>
       <c r="W12" t="s">
+        <v>223</v>
+      </c>
+      <c r="X12" t="s">
+        <v>224</v>
+      </c>
+      <c r="Y12" t="s">
         <v>222</v>
       </c>
-      <c r="X12" t="s">
-        <v>223</v>
-      </c>
-      <c r="Y12" t="s">
-        <v>221</v>
-      </c>
       <c r="Z12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AA12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AB12" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AC12" t="s">
         <v>160</v>
@@ -3343,7 +3344,7 @@
         <v>70</v>
       </c>
       <c r="AL12" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AM12" t="s">
         <v>72</v>
@@ -3352,10 +3353,10 @@
         <v>73</v>
       </c>
       <c r="AO12" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AP12" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.3">
@@ -3366,58 +3367,58 @@
         <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E13" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F13" t="s">
         <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="I13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="J13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="L13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M13" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="N13" t="s">
         <v>55</v>
       </c>
       <c r="O13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P13" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="Q13" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="S13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="T13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="U13" t="s">
         <v>60</v>
@@ -3426,31 +3427,31 @@
         <v>60</v>
       </c>
       <c r="W13" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="X13" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="Y13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Z13" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AA13" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AB13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="AC13" t="s">
         <v>160</v>
       </c>
       <c r="AD13" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AE13" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AF13" t="s">
         <v>70</v>
@@ -3483,7 +3484,7 @@
         <v>49</v>
       </c>
       <c r="AP13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="14" spans="1:42" x14ac:dyDescent="0.3">
@@ -3494,34 +3495,34 @@
         <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F14" t="s">
         <v>47</v>
       </c>
       <c r="G14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H14" t="s">
         <v>49</v>
       </c>
       <c r="I14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K14" t="s">
         <v>63</v>
       </c>
       <c r="L14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M14" t="s">
         <v>86</v>
@@ -3530,7 +3531,7 @@
         <v>55</v>
       </c>
       <c r="O14" t="s">
-        <v>257</v>
+        <v>153</v>
       </c>
       <c r="P14" t="s">
         <v>258</v>
@@ -3649,16 +3650,16 @@
         <v>259</v>
       </c>
       <c r="L15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="N15" t="s">
         <v>55</v>
       </c>
       <c r="O15" t="s">
-        <v>257</v>
+        <v>153</v>
       </c>
       <c r="P15" t="s">
         <v>268</v>
@@ -3700,13 +3701,13 @@
         <v>274</v>
       </c>
       <c r="AC15" t="s">
-        <v>160</v>
+        <v>67</v>
       </c>
       <c r="AD15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AE15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AF15" t="s">
         <v>70</v>
@@ -3777,7 +3778,7 @@
         <v>107</v>
       </c>
       <c r="L16" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M16" t="s">
         <v>86</v>
@@ -3786,13 +3787,13 @@
         <v>55</v>
       </c>
       <c r="O16" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P16" t="s">
         <v>282</v>
       </c>
       <c r="Q16" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R16" t="s">
         <v>90</v>
@@ -3816,7 +3817,7 @@
         <v>94</v>
       </c>
       <c r="Y16" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Z16" t="s">
         <v>95</v>
@@ -3825,7 +3826,7 @@
         <v>273</v>
       </c>
       <c r="AB16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AC16" t="s">
         <v>160</v>
@@ -3905,7 +3906,7 @@
         <v>290</v>
       </c>
       <c r="L17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M17" t="s">
         <v>86</v>
@@ -3920,7 +3921,7 @@
         <v>108</v>
       </c>
       <c r="Q17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R17" t="s">
         <v>90</v>
@@ -3953,7 +3954,7 @@
         <v>273</v>
       </c>
       <c r="AB17" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AC17" t="s">
         <v>160</v>
@@ -4033,7 +4034,7 @@
         <v>290</v>
       </c>
       <c r="L18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M18" t="s">
         <v>54</v>
@@ -4048,7 +4049,7 @@
         <v>108</v>
       </c>
       <c r="Q18" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R18" t="s">
         <v>292</v>
@@ -4161,7 +4162,7 @@
         <v>306</v>
       </c>
       <c r="L19" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M19" t="s">
         <v>54</v>
@@ -4176,7 +4177,7 @@
         <v>307</v>
       </c>
       <c r="Q19" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R19" t="s">
         <v>142</v>

</xml_diff>

<commit_message>
📊 Actualizar CV_VU.xlsx — 25-03-2026, 10:00:27 a. m.
</commit_message>
<xml_diff>
--- a/datos/CV_VU.xlsx
+++ b/datos/CV_VU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F34CD0B-5A3D-40ED-A98A-0207545A63D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{75A0903B-B73F-4DE5-A41A-420504FF9BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="347">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -956,6 +956,111 @@
   </si>
   <si>
     <t>1015663</t>
+  </si>
+  <si>
+    <t>4137131-5</t>
+  </si>
+  <si>
+    <t>ARANCIBIA GAMBOA ROBERTO JAIME</t>
+  </si>
+  <si>
+    <t>10/08/1942</t>
+  </si>
+  <si>
+    <t>6132 - Pedro Aguirre Cerda - Santiago -CP</t>
+  </si>
+  <si>
+    <t>936398005 - 91368496</t>
+  </si>
+  <si>
+    <t>rarancibia430@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>21/03/2026</t>
+  </si>
+  <si>
+    <t>24/03/2026</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>45763</t>
+  </si>
+  <si>
+    <t>1015676</t>
+  </si>
+  <si>
+    <t>17680901-9</t>
+  </si>
+  <si>
+    <t>IBAÑEZ NUÑEZ CONSTANZA JANICE</t>
+  </si>
+  <si>
+    <t>09/09/1991</t>
+  </si>
+  <si>
+    <t>Renca</t>
+  </si>
+  <si>
+    <t>3176 - Renca - Santiago -CP</t>
+  </si>
+  <si>
+    <t>933158189</t>
+  </si>
+  <si>
+    <t>constanzajanice@gmaim.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>10.2</t>
+  </si>
+  <si>
+    <t>600000</t>
+  </si>
+  <si>
+    <t>5280000</t>
+  </si>
+  <si>
+    <t>146667</t>
+  </si>
+  <si>
+    <t>Valles De las Rosas</t>
+  </si>
+  <si>
+    <t>1-X-18</t>
+  </si>
+  <si>
+    <t>1015681</t>
+  </si>
+  <si>
+    <t>11399404-3</t>
+  </si>
+  <si>
+    <t>GUERRA LEIVA ANA EDELMIRA</t>
+  </si>
+  <si>
+    <t>24/09/1968</t>
+  </si>
+  <si>
+    <t>456 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>957359715</t>
+  </si>
+  <si>
+    <t>942854716</t>
+  </si>
+  <si>
+    <t>edelmiraguerraleiv@gmail.com - EDELMIRAGUERRALEIV@; ; ; ;</t>
+  </si>
+  <si>
+    <t>Nayaret Tatiana Puga Marchant</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>1015684</t>
   </si>
 </sst>
 </file>
@@ -1816,11 +1921,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP19"/>
+  <dimension ref="A1:AP22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="41" width="8" customWidth="1"/>
-    <col min="42" max="42" width="12" customWidth="1"/>
+    <col min="1" max="42" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.3">
@@ -4255,6 +4359,390 @@
         <v>311</v>
       </c>
     </row>
+    <row r="20" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" t="s">
+        <v>312</v>
+      </c>
+      <c r="D20" t="s">
+        <v>313</v>
+      </c>
+      <c r="E20" t="s">
+        <v>314</v>
+      </c>
+      <c r="F20" t="s">
+        <v>165</v>
+      </c>
+      <c r="G20" t="s">
+        <v>315</v>
+      </c>
+      <c r="H20" t="s">
+        <v>49</v>
+      </c>
+      <c r="I20" t="s">
+        <v>316</v>
+      </c>
+      <c r="J20" t="s">
+        <v>317</v>
+      </c>
+      <c r="K20" t="s">
+        <v>318</v>
+      </c>
+      <c r="L20" t="s">
+        <v>319</v>
+      </c>
+      <c r="M20" t="s">
+        <v>86</v>
+      </c>
+      <c r="N20" t="s">
+        <v>55</v>
+      </c>
+      <c r="O20" t="s">
+        <v>153</v>
+      </c>
+      <c r="P20" t="s">
+        <v>268</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>320</v>
+      </c>
+      <c r="R20" t="s">
+        <v>90</v>
+      </c>
+      <c r="S20" t="s">
+        <v>91</v>
+      </c>
+      <c r="T20" t="s">
+        <v>92</v>
+      </c>
+      <c r="U20" t="s">
+        <v>60</v>
+      </c>
+      <c r="V20" t="s">
+        <v>60</v>
+      </c>
+      <c r="W20" t="s">
+        <v>93</v>
+      </c>
+      <c r="X20" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>318</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>321</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>160</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM20" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO20" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP20" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="21" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" t="s">
+        <v>323</v>
+      </c>
+      <c r="D21" t="s">
+        <v>324</v>
+      </c>
+      <c r="E21" t="s">
+        <v>325</v>
+      </c>
+      <c r="F21" t="s">
+        <v>326</v>
+      </c>
+      <c r="G21" t="s">
+        <v>327</v>
+      </c>
+      <c r="H21" t="s">
+        <v>49</v>
+      </c>
+      <c r="I21" t="s">
+        <v>328</v>
+      </c>
+      <c r="J21" t="s">
+        <v>329</v>
+      </c>
+      <c r="K21" t="s">
+        <v>290</v>
+      </c>
+      <c r="L21" t="s">
+        <v>319</v>
+      </c>
+      <c r="M21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N21" t="s">
+        <v>55</v>
+      </c>
+      <c r="O21" t="s">
+        <v>239</v>
+      </c>
+      <c r="P21" t="s">
+        <v>282</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>198</v>
+      </c>
+      <c r="R21" t="s">
+        <v>209</v>
+      </c>
+      <c r="S21" t="s">
+        <v>209</v>
+      </c>
+      <c r="T21" t="s">
+        <v>209</v>
+      </c>
+      <c r="U21" t="s">
+        <v>60</v>
+      </c>
+      <c r="V21" t="s">
+        <v>60</v>
+      </c>
+      <c r="W21" t="s">
+        <v>330</v>
+      </c>
+      <c r="X21" t="s">
+        <v>331</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>290</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>332</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>143</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>333</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>160</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH21" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI21" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ21" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL21" t="s">
+        <v>334</v>
+      </c>
+      <c r="AM21" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN21" t="s">
+        <v>73</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>335</v>
+      </c>
+      <c r="AP21" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="22" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>337</v>
+      </c>
+      <c r="D22" t="s">
+        <v>338</v>
+      </c>
+      <c r="E22" t="s">
+        <v>339</v>
+      </c>
+      <c r="F22" t="s">
+        <v>47</v>
+      </c>
+      <c r="G22" t="s">
+        <v>340</v>
+      </c>
+      <c r="H22" t="s">
+        <v>341</v>
+      </c>
+      <c r="I22" t="s">
+        <v>342</v>
+      </c>
+      <c r="J22" t="s">
+        <v>343</v>
+      </c>
+      <c r="K22" t="s">
+        <v>319</v>
+      </c>
+      <c r="L22" t="s">
+        <v>319</v>
+      </c>
+      <c r="M22" t="s">
+        <v>86</v>
+      </c>
+      <c r="N22" t="s">
+        <v>55</v>
+      </c>
+      <c r="O22" t="s">
+        <v>153</v>
+      </c>
+      <c r="P22" t="s">
+        <v>344</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>320</v>
+      </c>
+      <c r="R22" t="s">
+        <v>90</v>
+      </c>
+      <c r="S22" t="s">
+        <v>91</v>
+      </c>
+      <c r="T22" t="s">
+        <v>92</v>
+      </c>
+      <c r="U22" t="s">
+        <v>60</v>
+      </c>
+      <c r="V22" t="s">
+        <v>60</v>
+      </c>
+      <c r="W22" t="s">
+        <v>93</v>
+      </c>
+      <c r="X22" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>319</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>345</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>321</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>160</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK22" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM22" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO22" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP22" t="s">
+        <v>346</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
📊 Actualizar CV_VU.xlsx — 26-03-2026, 11:53:59 a. m.
</commit_message>
<xml_diff>
--- a/datos/CV_VU.xlsx
+++ b/datos/CV_VU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A1CD6A8-DC73-44CC-97DE-9E2609E9A950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{61AB646D-0263-4BFE-864B-79838BFC6036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="373">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -502,84 +502,84 @@
     <t>76667</t>
   </si>
   <si>
+    <t>1015622</t>
+  </si>
+  <si>
+    <t>22318996-2</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ ESPINOZA ALONSO</t>
+  </si>
+  <si>
+    <t>19/04/1983</t>
+  </si>
+  <si>
+    <t>Pedro Aguirre Cerda</t>
+  </si>
+  <si>
+    <t>5455 - Pedro Aguirre Cerda - Santiago -CP</t>
+  </si>
+  <si>
+    <t>978737691</t>
+  </si>
+  <si>
+    <t>alonsorodriguezespinoza1904@gmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>11/03/2026</t>
+  </si>
+  <si>
+    <t>Nf Cartera</t>
+  </si>
+  <si>
+    <t>1000000</t>
+  </si>
+  <si>
+    <t>00/00/0000</t>
+  </si>
+  <si>
+    <t>Valle De La Memoria</t>
+  </si>
+  <si>
+    <t>Valle de la Memoria</t>
+  </si>
+  <si>
+    <t>3-BA-43</t>
+  </si>
+  <si>
+    <t>1015629</t>
+  </si>
+  <si>
+    <t>18190149-7</t>
+  </si>
+  <si>
+    <t>CAYUN HEREDIA KAREN ANDREA</t>
+  </si>
+  <si>
+    <t>03/02/1992</t>
+  </si>
+  <si>
+    <t>Huechuraba</t>
+  </si>
+  <si>
+    <t>228 - Huechuraba - Santiago -CP</t>
+  </si>
+  <si>
+    <t>920512919</t>
+  </si>
+  <si>
+    <t>920234538</t>
+  </si>
+  <si>
+    <t>KARENCAYUNHEREDIA@GMAIL.COM; ; ; ;</t>
+  </si>
+  <si>
+    <t>1347000</t>
+  </si>
+  <si>
     <t>ACTIVO PEND VALIDAR</t>
   </si>
   <si>
-    <t>1015622</t>
-  </si>
-  <si>
-    <t>22318996-2</t>
-  </si>
-  <si>
-    <t>RODRIGUEZ ESPINOZA ALONSO</t>
-  </si>
-  <si>
-    <t>19/04/1983</t>
-  </si>
-  <si>
-    <t>Pedro Aguirre Cerda</t>
-  </si>
-  <si>
-    <t>5455 - Pedro Aguirre Cerda - Santiago -CP</t>
-  </si>
-  <si>
-    <t>978737691</t>
-  </si>
-  <si>
-    <t>alonsorodriguezespinoza1904@gmail.com; ; ; ;</t>
-  </si>
-  <si>
-    <t>11/03/2026</t>
-  </si>
-  <si>
-    <t>Nf Cartera</t>
-  </si>
-  <si>
-    <t>1000000</t>
-  </si>
-  <si>
-    <t>00/00/0000</t>
-  </si>
-  <si>
-    <t>Valle De La Memoria</t>
-  </si>
-  <si>
-    <t>Valle de la Memoria</t>
-  </si>
-  <si>
-    <t>3-BA-43</t>
-  </si>
-  <si>
-    <t>1015629</t>
-  </si>
-  <si>
-    <t>18190149-7</t>
-  </si>
-  <si>
-    <t>CAYUN HEREDIA KAREN ANDREA</t>
-  </si>
-  <si>
-    <t>03/02/1992</t>
-  </si>
-  <si>
-    <t>Huechuraba</t>
-  </si>
-  <si>
-    <t>228 - Huechuraba - Santiago -CP</t>
-  </si>
-  <si>
-    <t>920512919</t>
-  </si>
-  <si>
-    <t>920234538</t>
-  </si>
-  <si>
-    <t>KARENCAYUNHEREDIA@GMAIL.COM; ; ; ;</t>
-  </si>
-  <si>
-    <t>1347000</t>
-  </si>
-  <si>
     <t>MIGRAR</t>
   </si>
   <si>
@@ -1033,6 +1033,48 @@
     <t>1015681</t>
   </si>
   <si>
+    <t>6839198-9</t>
+  </si>
+  <si>
+    <t>HERMOSILLA NORAMBUENA GRACIELA DEL CARMEN</t>
+  </si>
+  <si>
+    <t>05/01/1949</t>
+  </si>
+  <si>
+    <t>La Pintana</t>
+  </si>
+  <si>
+    <t>11122 - La Pintana - Santiago -CP</t>
+  </si>
+  <si>
+    <t>987418795</t>
+  </si>
+  <si>
+    <t>mana2010@live.cl; ; ; ;</t>
+  </si>
+  <si>
+    <t>25/03/2026</t>
+  </si>
+  <si>
+    <t>Nayaret Tatiana Puga Marchant</t>
+  </si>
+  <si>
+    <t>33.33</t>
+  </si>
+  <si>
+    <t>2000000</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>33898</t>
+  </si>
+  <si>
+    <t>1015683</t>
+  </si>
+  <si>
     <t>11399404-3</t>
   </si>
   <si>
@@ -1054,13 +1096,49 @@
     <t>edelmiraguerraleiv@gmail.com - EDELMIRAGUERRALEIV@; ; ; ;</t>
   </si>
   <si>
-    <t>Nayaret Tatiana Puga Marchant</t>
-  </si>
-  <si>
     <t>24</t>
   </si>
   <si>
     <t>1015684</t>
+  </si>
+  <si>
+    <t>10740648-4</t>
+  </si>
+  <si>
+    <t>GALLARDO CONTRERAS SILVIA ISABEL</t>
+  </si>
+  <si>
+    <t>28/10/1967</t>
+  </si>
+  <si>
+    <t>485 - Quilicura - Santiago -CP</t>
+  </si>
+  <si>
+    <t>964469773</t>
+  </si>
+  <si>
+    <t>975782194</t>
+  </si>
+  <si>
+    <t>sigallardo28@hotmail.com; ; ; ;</t>
+  </si>
+  <si>
+    <t>34.01</t>
+  </si>
+  <si>
+    <t>3880000</t>
+  </si>
+  <si>
+    <t>107778</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2-AA-4</t>
+  </si>
+  <si>
+    <t>1015686</t>
   </si>
 </sst>
 </file>
@@ -1921,10 +1999,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP22"/>
+  <dimension ref="A1:AP24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="42" width="8" customWidth="1"/>
+    <col min="1" max="41" width="8" customWidth="1"/>
+    <col min="42" max="42" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.3">
@@ -2781,7 +2860,7 @@
         <v>159</v>
       </c>
       <c r="AC7" t="s">
-        <v>160</v>
+        <v>67</v>
       </c>
       <c r="AD7" t="s">
         <v>127</v>
@@ -2820,7 +2899,7 @@
         <v>49</v>
       </c>
       <c r="AP7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.3">
@@ -2831,34 +2910,34 @@
         <v>43</v>
       </c>
       <c r="C8" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" t="s">
         <v>162</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>163</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>164</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>165</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>166</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
+        <v>166</v>
+      </c>
+      <c r="J8" t="s">
         <v>167</v>
-      </c>
-      <c r="I8" t="s">
-        <v>167</v>
-      </c>
-      <c r="J8" t="s">
-        <v>168</v>
       </c>
       <c r="K8" t="s">
         <v>53</v>
       </c>
       <c r="L8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M8" t="s">
         <v>54</v>
@@ -2870,19 +2949,19 @@
         <v>49</v>
       </c>
       <c r="P8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q8" t="s">
         <v>65</v>
       </c>
       <c r="R8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="S8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="U8" t="s">
         <v>60</v>
@@ -2897,46 +2976,46 @@
         <v>60</v>
       </c>
       <c r="Y8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Z8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AA8" t="s">
         <v>93</v>
       </c>
       <c r="AB8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AC8" t="s">
-        <v>160</v>
+        <v>67</v>
       </c>
       <c r="AD8" t="s">
         <v>68</v>
       </c>
       <c r="AE8" t="s">
+        <v>172</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI8" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL8" t="s">
         <v>173</v>
-      </c>
-      <c r="AF8" t="s">
-        <v>70</v>
-      </c>
-      <c r="AG8" t="s">
-        <v>70</v>
-      </c>
-      <c r="AH8" t="s">
-        <v>70</v>
-      </c>
-      <c r="AI8" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ8" t="s">
-        <v>70</v>
-      </c>
-      <c r="AK8" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL8" t="s">
-        <v>174</v>
       </c>
       <c r="AM8" t="s">
         <v>72</v>
@@ -2945,10 +3024,10 @@
         <v>73</v>
       </c>
       <c r="AO8" t="s">
+        <v>174</v>
+      </c>
+      <c r="AP8" t="s">
         <v>175</v>
-      </c>
-      <c r="AP8" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.3">
@@ -2959,34 +3038,34 @@
         <v>43</v>
       </c>
       <c r="C9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D9" t="s">
         <v>177</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>178</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>179</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>180</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>181</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>182</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>183</v>
-      </c>
-      <c r="J9" t="s">
-        <v>184</v>
       </c>
       <c r="K9" t="s">
         <v>53</v>
       </c>
       <c r="L9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M9" t="s">
         <v>54</v>
@@ -2998,19 +3077,19 @@
         <v>49</v>
       </c>
       <c r="P9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q9" t="s">
         <v>65</v>
       </c>
       <c r="R9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="S9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="T9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="U9" t="s">
         <v>60</v>
@@ -3025,19 +3104,19 @@
         <v>60</v>
       </c>
       <c r="Y9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Z9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AA9" t="s">
         <v>93</v>
       </c>
       <c r="AB9" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC9" t="s">
         <v>185</v>
-      </c>
-      <c r="AC9" t="s">
-        <v>160</v>
       </c>
       <c r="AD9" t="s">
         <v>68</v>
@@ -3114,7 +3193,7 @@
         <v>196</v>
       </c>
       <c r="L10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M10" t="s">
         <v>86</v>
@@ -3242,7 +3321,7 @@
         <v>156</v>
       </c>
       <c r="L11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M11" t="s">
         <v>54</v>
@@ -3281,7 +3360,7 @@
         <v>210</v>
       </c>
       <c r="Y11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Z11" t="s">
         <v>211</v>
@@ -3421,13 +3500,13 @@
         <v>227</v>
       </c>
       <c r="AC12" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD12" t="s">
         <v>68</v>
       </c>
       <c r="AE12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AF12" t="s">
         <v>70</v>
@@ -3549,7 +3628,7 @@
         <v>249</v>
       </c>
       <c r="AC13" t="s">
-        <v>160</v>
+        <v>67</v>
       </c>
       <c r="AD13" t="s">
         <v>250</v>
@@ -3677,7 +3756,7 @@
         <v>260</v>
       </c>
       <c r="AC14" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD14" t="s">
         <v>98</v>
@@ -3933,7 +4012,7 @@
         <v>200</v>
       </c>
       <c r="AC16" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD16" t="s">
         <v>98</v>
@@ -4061,7 +4140,7 @@
         <v>200</v>
       </c>
       <c r="AC17" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD17" t="s">
         <v>98</v>
@@ -4189,7 +4268,7 @@
         <v>297</v>
       </c>
       <c r="AC18" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD18" t="s">
         <v>68</v>
@@ -4317,13 +4396,13 @@
         <v>310</v>
       </c>
       <c r="AC19" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD19" t="s">
         <v>68</v>
       </c>
       <c r="AE19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AF19" t="s">
         <v>70</v>
@@ -4376,7 +4455,7 @@
         <v>314</v>
       </c>
       <c r="F20" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G20" t="s">
         <v>315</v>
@@ -4445,7 +4524,7 @@
         <v>321</v>
       </c>
       <c r="AC20" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD20" t="s">
         <v>98</v>
@@ -4573,7 +4652,7 @@
         <v>333</v>
       </c>
       <c r="AC21" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD21" t="s">
         <v>68</v>
@@ -4632,13 +4711,13 @@
         <v>339</v>
       </c>
       <c r="F22" t="s">
-        <v>47</v>
+        <v>340</v>
       </c>
       <c r="G22" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H22" t="s">
-        <v>341</v>
+        <v>49</v>
       </c>
       <c r="I22" t="s">
         <v>342</v>
@@ -4647,10 +4726,10 @@
         <v>343</v>
       </c>
       <c r="K22" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="L22" t="s">
-        <v>319</v>
+        <v>344</v>
       </c>
       <c r="M22" t="s">
         <v>86</v>
@@ -4662,7 +4741,7 @@
         <v>153</v>
       </c>
       <c r="P22" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="Q22" t="s">
         <v>320</v>
@@ -4683,25 +4762,25 @@
         <v>60</v>
       </c>
       <c r="W22" t="s">
-        <v>93</v>
+        <v>346</v>
       </c>
       <c r="X22" t="s">
-        <v>94</v>
+        <v>170</v>
       </c>
       <c r="Y22" t="s">
-        <v>319</v>
+        <v>344</v>
       </c>
       <c r="Z22" t="s">
-        <v>95</v>
+        <v>347</v>
       </c>
       <c r="AA22" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="AB22" t="s">
-        <v>321</v>
+        <v>349</v>
       </c>
       <c r="AC22" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="AD22" t="s">
         <v>98</v>
@@ -4740,7 +4819,263 @@
         <v>49</v>
       </c>
       <c r="AP22" t="s">
-        <v>346</v>
+        <v>350</v>
+      </c>
+    </row>
+    <row r="23" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>351</v>
+      </c>
+      <c r="D23" t="s">
+        <v>352</v>
+      </c>
+      <c r="E23" t="s">
+        <v>353</v>
+      </c>
+      <c r="F23" t="s">
+        <v>47</v>
+      </c>
+      <c r="G23" t="s">
+        <v>354</v>
+      </c>
+      <c r="H23" t="s">
+        <v>355</v>
+      </c>
+      <c r="I23" t="s">
+        <v>356</v>
+      </c>
+      <c r="J23" t="s">
+        <v>357</v>
+      </c>
+      <c r="K23" t="s">
+        <v>319</v>
+      </c>
+      <c r="L23" t="s">
+        <v>319</v>
+      </c>
+      <c r="M23" t="s">
+        <v>86</v>
+      </c>
+      <c r="N23" t="s">
+        <v>55</v>
+      </c>
+      <c r="O23" t="s">
+        <v>153</v>
+      </c>
+      <c r="P23" t="s">
+        <v>345</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>320</v>
+      </c>
+      <c r="R23" t="s">
+        <v>90</v>
+      </c>
+      <c r="S23" t="s">
+        <v>91</v>
+      </c>
+      <c r="T23" t="s">
+        <v>92</v>
+      </c>
+      <c r="U23" t="s">
+        <v>60</v>
+      </c>
+      <c r="V23" t="s">
+        <v>60</v>
+      </c>
+      <c r="W23" t="s">
+        <v>93</v>
+      </c>
+      <c r="X23" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>319</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>358</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>321</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK23" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM23" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO23" t="s">
+        <v>49</v>
+      </c>
+      <c r="AP23" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="24" spans="1:42" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>360</v>
+      </c>
+      <c r="D24" t="s">
+        <v>361</v>
+      </c>
+      <c r="E24" t="s">
+        <v>362</v>
+      </c>
+      <c r="F24" t="s">
+        <v>47</v>
+      </c>
+      <c r="G24" t="s">
+        <v>363</v>
+      </c>
+      <c r="H24" t="s">
+        <v>364</v>
+      </c>
+      <c r="I24" t="s">
+        <v>365</v>
+      </c>
+      <c r="J24" t="s">
+        <v>366</v>
+      </c>
+      <c r="K24" t="s">
+        <v>344</v>
+      </c>
+      <c r="L24" t="s">
+        <v>344</v>
+      </c>
+      <c r="M24" t="s">
+        <v>54</v>
+      </c>
+      <c r="N24" t="s">
+        <v>55</v>
+      </c>
+      <c r="O24" t="s">
+        <v>49</v>
+      </c>
+      <c r="P24" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>198</v>
+      </c>
+      <c r="R24" t="s">
+        <v>209</v>
+      </c>
+      <c r="S24" t="s">
+        <v>209</v>
+      </c>
+      <c r="T24" t="s">
+        <v>209</v>
+      </c>
+      <c r="U24" t="s">
+        <v>60</v>
+      </c>
+      <c r="V24" t="s">
+        <v>60</v>
+      </c>
+      <c r="W24" t="s">
+        <v>367</v>
+      </c>
+      <c r="X24" t="s">
+        <v>347</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>344</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>368</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>199</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>369</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI24" t="s">
+        <v>49</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>70</v>
+      </c>
+      <c r="AL24" t="s">
+        <v>71</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>72</v>
+      </c>
+      <c r="AN24" t="s">
+        <v>370</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>371</v>
+      </c>
+      <c r="AP24" t="s">
+        <v>372</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Actualizar CV_VU.xlsx — 30-03-2026, 1:53:47 p. m.
</commit_message>
<xml_diff>
--- a/datos/CV_VU.xlsx
+++ b/datos/CV_VU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61AB646D-0263-4BFE-864B-79838BFC6036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{66871571-4161-4DC0-9585-70410936B723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="340">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -505,90 +505,30 @@
     <t>1015622</t>
   </si>
   <si>
-    <t>22318996-2</t>
-  </si>
-  <si>
-    <t>RODRIGUEZ ESPINOZA ALONSO</t>
-  </si>
-  <si>
-    <t>19/04/1983</t>
-  </si>
-  <si>
     <t>Pedro Aguirre Cerda</t>
   </si>
   <si>
-    <t>5455 - Pedro Aguirre Cerda - Santiago -CP</t>
-  </si>
-  <si>
-    <t>978737691</t>
-  </si>
-  <si>
-    <t>alonsorodriguezespinoza1904@gmail.com; ; ; ;</t>
-  </si>
-  <si>
     <t>11/03/2026</t>
   </si>
   <si>
-    <t>Nf Cartera</t>
-  </si>
-  <si>
     <t>1000000</t>
   </si>
   <si>
-    <t>00/00/0000</t>
-  </si>
-  <si>
     <t>Valle De La Memoria</t>
   </si>
   <si>
-    <t>Valle de la Memoria</t>
-  </si>
-  <si>
-    <t>3-BA-43</t>
-  </si>
-  <si>
-    <t>1015629</t>
-  </si>
-  <si>
-    <t>18190149-7</t>
-  </si>
-  <si>
-    <t>CAYUN HEREDIA KAREN ANDREA</t>
-  </si>
-  <si>
-    <t>03/02/1992</t>
-  </si>
-  <si>
-    <t>Huechuraba</t>
-  </si>
-  <si>
-    <t>228 - Huechuraba - Santiago -CP</t>
-  </si>
-  <si>
-    <t>920512919</t>
-  </si>
-  <si>
-    <t>920234538</t>
-  </si>
-  <si>
-    <t>KARENCAYUNHEREDIA@GMAIL.COM; ; ; ;</t>
-  </si>
-  <si>
-    <t>1347000</t>
-  </si>
-  <si>
     <t>ACTIVO PEND VALIDAR</t>
   </si>
   <si>
     <t>MIGRAR</t>
   </si>
   <si>
+    <t>9</t>
+  </si>
+  <si>
     <t>SIN ASIGNAR</t>
   </si>
   <si>
-    <t>1015631</t>
-  </si>
-  <si>
     <t>10033214-0</t>
   </si>
   <si>
@@ -1100,45 +1040,6 @@
   </si>
   <si>
     <t>1015684</t>
-  </si>
-  <si>
-    <t>10740648-4</t>
-  </si>
-  <si>
-    <t>GALLARDO CONTRERAS SILVIA ISABEL</t>
-  </si>
-  <si>
-    <t>28/10/1967</t>
-  </si>
-  <si>
-    <t>485 - Quilicura - Santiago -CP</t>
-  </si>
-  <si>
-    <t>964469773</t>
-  </si>
-  <si>
-    <t>975782194</t>
-  </si>
-  <si>
-    <t>sigallardo28@hotmail.com; ; ; ;</t>
-  </si>
-  <si>
-    <t>34.01</t>
-  </si>
-  <si>
-    <t>3880000</t>
-  </si>
-  <si>
-    <t>107778</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>2-AA-4</t>
-  </si>
-  <si>
-    <t>1015686</t>
   </si>
 </sst>
 </file>
@@ -1999,7 +1900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP24"/>
+  <dimension ref="A1:AP21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="41" width="8" customWidth="1"/>
@@ -2910,58 +2811,58 @@
         <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="D8" t="s">
+        <v>170</v>
+      </c>
+      <c r="E8" t="s">
+        <v>171</v>
+      </c>
+      <c r="F8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" t="s">
+        <v>172</v>
+      </c>
+      <c r="H8" t="s">
+        <v>173</v>
+      </c>
+      <c r="I8" t="s">
+        <v>174</v>
+      </c>
+      <c r="J8" t="s">
+        <v>175</v>
+      </c>
+      <c r="K8" t="s">
+        <v>176</v>
+      </c>
+      <c r="L8" t="s">
         <v>162</v>
       </c>
-      <c r="E8" t="s">
-        <v>163</v>
-      </c>
-      <c r="F8" t="s">
-        <v>164</v>
-      </c>
-      <c r="G8" t="s">
-        <v>165</v>
-      </c>
-      <c r="H8" t="s">
-        <v>166</v>
-      </c>
-      <c r="I8" t="s">
-        <v>166</v>
-      </c>
-      <c r="J8" t="s">
-        <v>167</v>
-      </c>
-      <c r="K8" t="s">
-        <v>53</v>
-      </c>
-      <c r="L8" t="s">
-        <v>168</v>
-      </c>
       <c r="M8" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="N8" t="s">
         <v>55</v>
       </c>
       <c r="O8" t="s">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="P8" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="Q8" t="s">
-        <v>65</v>
+        <v>178</v>
       </c>
       <c r="R8" t="s">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="S8" t="s">
-        <v>170</v>
+        <v>91</v>
       </c>
       <c r="T8" t="s">
-        <v>170</v>
+        <v>92</v>
       </c>
       <c r="U8" t="s">
         <v>60</v>
@@ -2970,31 +2871,31 @@
         <v>60</v>
       </c>
       <c r="W8" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="X8" t="s">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="Y8" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="Z8" t="s">
-        <v>170</v>
+        <v>95</v>
       </c>
       <c r="AA8" t="s">
-        <v>93</v>
+        <v>179</v>
       </c>
       <c r="AB8" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="AC8" t="s">
         <v>67</v>
       </c>
       <c r="AD8" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AE8" t="s">
-        <v>172</v>
+        <v>86</v>
       </c>
       <c r="AF8" t="s">
         <v>70</v>
@@ -3015,19 +2916,19 @@
         <v>70</v>
       </c>
       <c r="AL8" t="s">
-        <v>173</v>
+        <v>49</v>
       </c>
       <c r="AM8" t="s">
         <v>72</v>
       </c>
       <c r="AN8" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="AO8" t="s">
-        <v>174</v>
+        <v>49</v>
       </c>
       <c r="AP8" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.3">
@@ -3038,34 +2939,34 @@
         <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D9" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="E9" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F9" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="G9" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="H9" t="s">
-        <v>181</v>
+        <v>49</v>
       </c>
       <c r="I9" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="J9" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="K9" t="s">
-        <v>53</v>
+        <v>156</v>
       </c>
       <c r="L9" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="M9" t="s">
         <v>54</v>
@@ -3074,22 +2975,22 @@
         <v>55</v>
       </c>
       <c r="O9" t="s">
-        <v>49</v>
+        <v>136</v>
       </c>
       <c r="P9" t="s">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="Q9" t="s">
-        <v>65</v>
+        <v>178</v>
       </c>
       <c r="R9" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="S9" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="T9" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="U9" t="s">
         <v>60</v>
@@ -3098,25 +2999,25 @@
         <v>60</v>
       </c>
       <c r="W9" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="X9" t="s">
-        <v>60</v>
+        <v>190</v>
       </c>
       <c r="Y9" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="Z9" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="AA9" t="s">
-        <v>93</v>
+        <v>192</v>
       </c>
       <c r="AB9" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="AC9" t="s">
-        <v>185</v>
+        <v>67</v>
       </c>
       <c r="AD9" t="s">
         <v>68</v>
@@ -3143,19 +3044,19 @@
         <v>70</v>
       </c>
       <c r="AL9" t="s">
-        <v>186</v>
+        <v>166</v>
       </c>
       <c r="AM9" t="s">
         <v>72</v>
       </c>
       <c r="AN9" t="s">
-        <v>49</v>
+        <v>167</v>
       </c>
       <c r="AO9" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="AP9" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.3">
@@ -3166,58 +3067,58 @@
         <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D10" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="E10" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="F10" t="s">
         <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="H10" t="s">
-        <v>193</v>
+        <v>49</v>
       </c>
       <c r="I10" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="J10" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="K10" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="L10" t="s">
-        <v>168</v>
+        <v>202</v>
       </c>
       <c r="M10" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="N10" t="s">
         <v>55</v>
       </c>
       <c r="O10" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="P10" t="s">
-        <v>197</v>
+        <v>57</v>
       </c>
       <c r="Q10" t="s">
-        <v>198</v>
+        <v>109</v>
       </c>
       <c r="R10" t="s">
-        <v>90</v>
+        <v>139</v>
       </c>
       <c r="S10" t="s">
-        <v>91</v>
+        <v>139</v>
       </c>
       <c r="T10" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
       <c r="U10" t="s">
         <v>60</v>
@@ -3226,31 +3127,31 @@
         <v>60</v>
       </c>
       <c r="W10" t="s">
-        <v>93</v>
+        <v>203</v>
       </c>
       <c r="X10" t="s">
-        <v>94</v>
+        <v>204</v>
       </c>
       <c r="Y10" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="Z10" t="s">
-        <v>95</v>
+        <v>205</v>
       </c>
       <c r="AA10" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="AB10" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="AC10" t="s">
-        <v>67</v>
+        <v>165</v>
       </c>
       <c r="AD10" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="AE10" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="AF10" t="s">
         <v>70</v>
@@ -3271,19 +3172,19 @@
         <v>70</v>
       </c>
       <c r="AL10" t="s">
-        <v>49</v>
+        <v>208</v>
       </c>
       <c r="AM10" t="s">
         <v>72</v>
       </c>
       <c r="AN10" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="AO10" t="s">
-        <v>49</v>
+        <v>209</v>
       </c>
       <c r="AP10" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.3">
@@ -3294,58 +3195,58 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="D11" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="E11" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="F11" t="s">
-        <v>205</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="H11" t="s">
-        <v>49</v>
+        <v>215</v>
       </c>
       <c r="I11" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="J11" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="K11" t="s">
-        <v>156</v>
+        <v>201</v>
       </c>
       <c r="L11" t="s">
-        <v>168</v>
+        <v>217</v>
       </c>
       <c r="M11" t="s">
-        <v>54</v>
+        <v>218</v>
       </c>
       <c r="N11" t="s">
         <v>55</v>
       </c>
       <c r="O11" t="s">
-        <v>136</v>
+        <v>219</v>
       </c>
       <c r="P11" t="s">
-        <v>137</v>
+        <v>220</v>
       </c>
       <c r="Q11" t="s">
-        <v>198</v>
+        <v>178</v>
       </c>
       <c r="R11" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="S11" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="T11" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="U11" t="s">
         <v>60</v>
@@ -3354,31 +3255,31 @@
         <v>60</v>
       </c>
       <c r="W11" t="s">
-        <v>93</v>
+        <v>224</v>
       </c>
       <c r="X11" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="Y11" t="s">
-        <v>168</v>
+        <v>226</v>
       </c>
       <c r="Z11" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="AA11" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="AB11" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="AC11" t="s">
         <v>67</v>
       </c>
       <c r="AD11" t="s">
-        <v>68</v>
+        <v>230</v>
       </c>
       <c r="AE11" t="s">
-        <v>69</v>
+        <v>218</v>
       </c>
       <c r="AF11" t="s">
         <v>70</v>
@@ -3399,7 +3300,7 @@
         <v>70</v>
       </c>
       <c r="AL11" t="s">
-        <v>186</v>
+        <v>49</v>
       </c>
       <c r="AM11" t="s">
         <v>72</v>
@@ -3408,10 +3309,10 @@
         <v>49</v>
       </c>
       <c r="AO11" t="s">
-        <v>187</v>
+        <v>49</v>
       </c>
       <c r="AP11" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.3">
@@ -3422,58 +3323,58 @@
         <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>215</v>
+        <v>232</v>
       </c>
       <c r="D12" t="s">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="E12" t="s">
-        <v>217</v>
+        <v>234</v>
       </c>
       <c r="F12" t="s">
         <v>47</v>
       </c>
       <c r="G12" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
       <c r="H12" t="s">
         <v>49</v>
       </c>
       <c r="I12" t="s">
-        <v>219</v>
+        <v>236</v>
       </c>
       <c r="J12" t="s">
-        <v>220</v>
+        <v>237</v>
       </c>
       <c r="K12" t="s">
-        <v>221</v>
+        <v>63</v>
       </c>
       <c r="L12" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="M12" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="N12" t="s">
         <v>55</v>
       </c>
       <c r="O12" t="s">
-        <v>56</v>
+        <v>153</v>
       </c>
       <c r="P12" t="s">
-        <v>57</v>
+        <v>238</v>
       </c>
       <c r="Q12" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="R12" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="S12" t="s">
-        <v>139</v>
+        <v>91</v>
       </c>
       <c r="T12" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="U12" t="s">
         <v>60</v>
@@ -3482,31 +3383,31 @@
         <v>60</v>
       </c>
       <c r="W12" t="s">
-        <v>223</v>
+        <v>93</v>
       </c>
       <c r="X12" t="s">
-        <v>224</v>
+        <v>94</v>
       </c>
       <c r="Y12" t="s">
-        <v>222</v>
+        <v>239</v>
       </c>
       <c r="Z12" t="s">
-        <v>225</v>
+        <v>95</v>
       </c>
       <c r="AA12" t="s">
-        <v>226</v>
+        <v>96</v>
       </c>
       <c r="AB12" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="AC12" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="AD12" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AE12" t="s">
-        <v>172</v>
+        <v>86</v>
       </c>
       <c r="AF12" t="s">
         <v>70</v>
@@ -3527,19 +3428,19 @@
         <v>70</v>
       </c>
       <c r="AL12" t="s">
-        <v>228</v>
+        <v>49</v>
       </c>
       <c r="AM12" t="s">
         <v>72</v>
       </c>
       <c r="AN12" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="AO12" t="s">
-        <v>229</v>
+        <v>49</v>
       </c>
       <c r="AP12" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.3">
@@ -3550,58 +3451,58 @@
         <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="D13" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="E13" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="F13" t="s">
         <v>47</v>
       </c>
       <c r="G13" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="H13" t="s">
-        <v>235</v>
+        <v>49</v>
       </c>
       <c r="I13" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="J13" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="K13" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="L13" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="M13" t="s">
-        <v>238</v>
+        <v>218</v>
       </c>
       <c r="N13" t="s">
         <v>55</v>
       </c>
       <c r="O13" t="s">
-        <v>239</v>
+        <v>153</v>
       </c>
       <c r="P13" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="Q13" t="s">
-        <v>198</v>
+        <v>89</v>
       </c>
       <c r="R13" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="S13" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="T13" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="U13" t="s">
         <v>60</v>
@@ -3610,31 +3511,31 @@
         <v>60</v>
       </c>
       <c r="W13" t="s">
-        <v>244</v>
+        <v>93</v>
       </c>
       <c r="X13" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="Y13" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="Z13" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="AA13" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="AB13" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AC13" t="s">
         <v>67</v>
       </c>
       <c r="AD13" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="AE13" t="s">
-        <v>238</v>
+        <v>218</v>
       </c>
       <c r="AF13" t="s">
         <v>70</v>
@@ -3667,7 +3568,7 @@
         <v>49</v>
       </c>
       <c r="AP13" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:42" x14ac:dyDescent="0.3">
@@ -3678,34 +3579,34 @@
         <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D14" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="E14" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="F14" t="s">
         <v>47</v>
       </c>
       <c r="G14" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="H14" t="s">
         <v>49</v>
       </c>
       <c r="I14" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="J14" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="K14" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="L14" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="M14" t="s">
         <v>86</v>
@@ -3714,13 +3615,13 @@
         <v>55</v>
       </c>
       <c r="O14" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="P14" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="Q14" t="s">
-        <v>138</v>
+        <v>178</v>
       </c>
       <c r="R14" t="s">
         <v>90</v>
@@ -3744,19 +3645,19 @@
         <v>94</v>
       </c>
       <c r="Y14" t="s">
-        <v>259</v>
+        <v>217</v>
       </c>
       <c r="Z14" t="s">
         <v>95</v>
       </c>
       <c r="AA14" t="s">
-        <v>96</v>
+        <v>253</v>
       </c>
       <c r="AB14" t="s">
-        <v>260</v>
+        <v>180</v>
       </c>
       <c r="AC14" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="AD14" t="s">
         <v>98</v>
@@ -3795,7 +3696,7 @@
         <v>49</v>
       </c>
       <c r="AP14" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.3">
@@ -3806,58 +3707,58 @@
         <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D15" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E15" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="F15" t="s">
         <v>47</v>
       </c>
       <c r="G15" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="H15" t="s">
-        <v>49</v>
+        <v>268</v>
       </c>
       <c r="I15" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="J15" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="K15" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="L15" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="M15" t="s">
-        <v>238</v>
+        <v>86</v>
       </c>
       <c r="N15" t="s">
         <v>55</v>
       </c>
       <c r="O15" t="s">
-        <v>153</v>
+        <v>87</v>
       </c>
       <c r="P15" t="s">
-        <v>268</v>
+        <v>108</v>
       </c>
       <c r="Q15" t="s">
-        <v>89</v>
+        <v>178</v>
       </c>
       <c r="R15" t="s">
-        <v>269</v>
+        <v>90</v>
       </c>
       <c r="S15" t="s">
-        <v>270</v>
+        <v>91</v>
       </c>
       <c r="T15" t="s">
-        <v>270</v>
+        <v>92</v>
       </c>
       <c r="U15" t="s">
         <v>60</v>
@@ -3869,28 +3770,28 @@
         <v>93</v>
       </c>
       <c r="X15" t="s">
-        <v>271</v>
+        <v>94</v>
       </c>
       <c r="Y15" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="Z15" t="s">
-        <v>272</v>
+        <v>95</v>
       </c>
       <c r="AA15" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="AB15" t="s">
-        <v>274</v>
+        <v>180</v>
       </c>
       <c r="AC15" t="s">
         <v>67</v>
       </c>
       <c r="AD15" t="s">
-        <v>250</v>
+        <v>98</v>
       </c>
       <c r="AE15" t="s">
-        <v>238</v>
+        <v>86</v>
       </c>
       <c r="AF15" t="s">
         <v>70</v>
@@ -3923,7 +3824,7 @@
         <v>49</v>
       </c>
       <c r="AP15" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.3">
@@ -3934,58 +3835,58 @@
         <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="D16" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="E16" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="F16" t="s">
         <v>47</v>
       </c>
       <c r="G16" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="H16" t="s">
-        <v>49</v>
+        <v>268</v>
       </c>
       <c r="I16" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="J16" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="K16" t="s">
-        <v>107</v>
+        <v>270</v>
       </c>
       <c r="L16" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="M16" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="N16" t="s">
         <v>55</v>
       </c>
       <c r="O16" t="s">
-        <v>239</v>
+        <v>87</v>
       </c>
       <c r="P16" t="s">
-        <v>282</v>
+        <v>108</v>
       </c>
       <c r="Q16" t="s">
-        <v>198</v>
+        <v>178</v>
       </c>
       <c r="R16" t="s">
-        <v>90</v>
+        <v>272</v>
       </c>
       <c r="S16" t="s">
-        <v>91</v>
+        <v>272</v>
       </c>
       <c r="T16" t="s">
-        <v>92</v>
+        <v>272</v>
       </c>
       <c r="U16" t="s">
         <v>60</v>
@@ -3994,31 +3895,31 @@
         <v>60</v>
       </c>
       <c r="W16" t="s">
-        <v>93</v>
+        <v>273</v>
       </c>
       <c r="X16" t="s">
-        <v>94</v>
+        <v>274</v>
       </c>
       <c r="Y16" t="s">
-        <v>237</v>
+        <v>275</v>
       </c>
       <c r="Z16" t="s">
-        <v>95</v>
+        <v>276</v>
       </c>
       <c r="AA16" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="AB16" t="s">
-        <v>200</v>
+        <v>277</v>
       </c>
       <c r="AC16" t="s">
-        <v>185</v>
+        <v>67</v>
       </c>
       <c r="AD16" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="AE16" t="s">
-        <v>86</v>
+        <v>278</v>
       </c>
       <c r="AF16" t="s">
         <v>70</v>
@@ -4039,19 +3940,19 @@
         <v>70</v>
       </c>
       <c r="AL16" t="s">
-        <v>49</v>
+        <v>166</v>
       </c>
       <c r="AM16" t="s">
         <v>72</v>
       </c>
       <c r="AN16" t="s">
-        <v>49</v>
+        <v>167</v>
       </c>
       <c r="AO16" t="s">
-        <v>49</v>
+        <v>168</v>
       </c>
       <c r="AP16" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
     </row>
     <row r="17" spans="1:42" x14ac:dyDescent="0.3">
@@ -4062,37 +3963,37 @@
         <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D17" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E17" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="F17" t="s">
         <v>47</v>
       </c>
       <c r="G17" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="H17" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="I17" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="J17" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="K17" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="L17" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="M17" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="N17" t="s">
         <v>55</v>
@@ -4101,19 +4002,19 @@
         <v>87</v>
       </c>
       <c r="P17" t="s">
-        <v>108</v>
+        <v>287</v>
       </c>
       <c r="Q17" t="s">
-        <v>198</v>
+        <v>178</v>
       </c>
       <c r="R17" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="S17" t="s">
-        <v>91</v>
+        <v>142</v>
       </c>
       <c r="T17" t="s">
-        <v>92</v>
+        <v>142</v>
       </c>
       <c r="U17" t="s">
         <v>60</v>
@@ -4122,31 +4023,31 @@
         <v>60</v>
       </c>
       <c r="W17" t="s">
-        <v>93</v>
+        <v>288</v>
       </c>
       <c r="X17" t="s">
-        <v>94</v>
+        <v>274</v>
       </c>
       <c r="Y17" t="s">
+        <v>286</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>289</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>253</v>
+      </c>
+      <c r="AB17" t="s">
         <v>290</v>
       </c>
-      <c r="Z17" t="s">
-        <v>95</v>
-      </c>
-      <c r="AA17" t="s">
-        <v>273</v>
-      </c>
-      <c r="AB17" t="s">
-        <v>200</v>
-      </c>
       <c r="AC17" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="AD17" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="AE17" t="s">
-        <v>86</v>
+        <v>164</v>
       </c>
       <c r="AF17" t="s">
         <v>70</v>
@@ -4167,16 +4068,16 @@
         <v>70</v>
       </c>
       <c r="AL17" t="s">
-        <v>49</v>
+        <v>166</v>
       </c>
       <c r="AM17" t="s">
         <v>72</v>
       </c>
       <c r="AN17" t="s">
-        <v>49</v>
+        <v>167</v>
       </c>
       <c r="AO17" t="s">
-        <v>49</v>
+        <v>168</v>
       </c>
       <c r="AP17" t="s">
         <v>291</v>
@@ -4190,58 +4091,58 @@
         <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="D18" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="E18" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="F18" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
       <c r="G18" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="H18" t="s">
-        <v>288</v>
+        <v>49</v>
       </c>
       <c r="I18" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="J18" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="K18" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="L18" t="s">
-        <v>237</v>
+        <v>299</v>
       </c>
       <c r="M18" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="N18" t="s">
         <v>55</v>
       </c>
       <c r="O18" t="s">
-        <v>87</v>
+        <v>153</v>
       </c>
       <c r="P18" t="s">
-        <v>108</v>
+        <v>248</v>
       </c>
       <c r="Q18" t="s">
-        <v>198</v>
+        <v>300</v>
       </c>
       <c r="R18" t="s">
-        <v>292</v>
+        <v>90</v>
       </c>
       <c r="S18" t="s">
-        <v>292</v>
+        <v>91</v>
       </c>
       <c r="T18" t="s">
-        <v>292</v>
+        <v>92</v>
       </c>
       <c r="U18" t="s">
         <v>60</v>
@@ -4250,31 +4151,31 @@
         <v>60</v>
       </c>
       <c r="W18" t="s">
-        <v>293</v>
+        <v>93</v>
       </c>
       <c r="X18" t="s">
-        <v>294</v>
+        <v>94</v>
       </c>
       <c r="Y18" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="Z18" t="s">
-        <v>296</v>
+        <v>95</v>
       </c>
       <c r="AA18" t="s">
-        <v>273</v>
+        <v>96</v>
       </c>
       <c r="AB18" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="AC18" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="AD18" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AE18" t="s">
-        <v>298</v>
+        <v>86</v>
       </c>
       <c r="AF18" t="s">
         <v>70</v>
@@ -4295,7 +4196,7 @@
         <v>70</v>
       </c>
       <c r="AL18" t="s">
-        <v>186</v>
+        <v>49</v>
       </c>
       <c r="AM18" t="s">
         <v>72</v>
@@ -4304,10 +4205,10 @@
         <v>49</v>
       </c>
       <c r="AO18" t="s">
-        <v>187</v>
+        <v>49</v>
       </c>
       <c r="AP18" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="19" spans="1:42" x14ac:dyDescent="0.3">
@@ -4318,34 +4219,34 @@
         <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D19" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E19" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F19" t="s">
-        <v>47</v>
+        <v>306</v>
       </c>
       <c r="G19" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="H19" t="s">
-        <v>304</v>
+        <v>49</v>
       </c>
       <c r="I19" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="J19" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="K19" t="s">
-        <v>306</v>
+        <v>270</v>
       </c>
       <c r="L19" t="s">
-        <v>237</v>
+        <v>299</v>
       </c>
       <c r="M19" t="s">
         <v>54</v>
@@ -4354,22 +4255,22 @@
         <v>55</v>
       </c>
       <c r="O19" t="s">
-        <v>87</v>
+        <v>219</v>
       </c>
       <c r="P19" t="s">
-        <v>307</v>
+        <v>262</v>
       </c>
       <c r="Q19" t="s">
-        <v>198</v>
+        <v>178</v>
       </c>
       <c r="R19" t="s">
-        <v>142</v>
+        <v>189</v>
       </c>
       <c r="S19" t="s">
-        <v>142</v>
+        <v>189</v>
       </c>
       <c r="T19" t="s">
-        <v>142</v>
+        <v>189</v>
       </c>
       <c r="U19" t="s">
         <v>60</v>
@@ -4378,31 +4279,31 @@
         <v>60</v>
       </c>
       <c r="W19" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="X19" t="s">
-        <v>294</v>
+        <v>311</v>
       </c>
       <c r="Y19" t="s">
-        <v>306</v>
+        <v>270</v>
       </c>
       <c r="Z19" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="AA19" t="s">
-        <v>273</v>
+        <v>143</v>
       </c>
       <c r="AB19" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="AC19" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="AD19" t="s">
         <v>68</v>
       </c>
       <c r="AE19" t="s">
-        <v>172</v>
+        <v>69</v>
       </c>
       <c r="AF19" t="s">
         <v>70</v>
@@ -4423,19 +4324,19 @@
         <v>70</v>
       </c>
       <c r="AL19" t="s">
-        <v>186</v>
+        <v>314</v>
       </c>
       <c r="AM19" t="s">
         <v>72</v>
       </c>
       <c r="AN19" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="AO19" t="s">
-        <v>187</v>
+        <v>315</v>
       </c>
       <c r="AP19" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" spans="1:42" x14ac:dyDescent="0.3">
@@ -4446,34 +4347,34 @@
         <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="D20" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="E20" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="F20" t="s">
-        <v>164</v>
+        <v>320</v>
       </c>
       <c r="G20" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="H20" t="s">
         <v>49</v>
       </c>
       <c r="I20" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J20" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="K20" t="s">
-        <v>318</v>
+        <v>298</v>
       </c>
       <c r="L20" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="M20" t="s">
         <v>86</v>
@@ -4485,10 +4386,10 @@
         <v>153</v>
       </c>
       <c r="P20" t="s">
-        <v>268</v>
+        <v>325</v>
       </c>
       <c r="Q20" t="s">
-        <v>320</v>
+        <v>300</v>
       </c>
       <c r="R20" t="s">
         <v>90</v>
@@ -4506,25 +4407,25 @@
         <v>60</v>
       </c>
       <c r="W20" t="s">
-        <v>93</v>
+        <v>326</v>
       </c>
       <c r="X20" t="s">
-        <v>94</v>
+        <v>163</v>
       </c>
       <c r="Y20" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="Z20" t="s">
-        <v>95</v>
+        <v>327</v>
       </c>
       <c r="AA20" t="s">
-        <v>96</v>
+        <v>328</v>
       </c>
       <c r="AB20" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="AC20" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="AD20" t="s">
         <v>98</v>
@@ -4563,7 +4464,7 @@
         <v>49</v>
       </c>
       <c r="AP20" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21" spans="1:42" x14ac:dyDescent="0.3">
@@ -4574,58 +4475,58 @@
         <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="D21" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="E21" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="F21" t="s">
-        <v>326</v>
+        <v>47</v>
       </c>
       <c r="G21" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="H21" t="s">
-        <v>49</v>
+        <v>335</v>
       </c>
       <c r="I21" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="J21" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="K21" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="L21" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="M21" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="N21" t="s">
         <v>55</v>
       </c>
       <c r="O21" t="s">
-        <v>239</v>
+        <v>153</v>
       </c>
       <c r="P21" t="s">
-        <v>282</v>
+        <v>325</v>
       </c>
       <c r="Q21" t="s">
-        <v>198</v>
+        <v>300</v>
       </c>
       <c r="R21" t="s">
-        <v>209</v>
+        <v>90</v>
       </c>
       <c r="S21" t="s">
-        <v>209</v>
+        <v>91</v>
       </c>
       <c r="T21" t="s">
-        <v>209</v>
+        <v>92</v>
       </c>
       <c r="U21" t="s">
         <v>60</v>
@@ -4634,31 +4535,31 @@
         <v>60</v>
       </c>
       <c r="W21" t="s">
-        <v>330</v>
+        <v>93</v>
       </c>
       <c r="X21" t="s">
-        <v>331</v>
+        <v>94</v>
       </c>
       <c r="Y21" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="Z21" t="s">
-        <v>332</v>
+        <v>95</v>
       </c>
       <c r="AA21" t="s">
-        <v>143</v>
+        <v>338</v>
       </c>
       <c r="AB21" t="s">
-        <v>333</v>
+        <v>301</v>
       </c>
       <c r="AC21" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="AD21" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="AE21" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="AF21" t="s">
         <v>70</v>
@@ -4679,403 +4580,19 @@
         <v>70</v>
       </c>
       <c r="AL21" t="s">
-        <v>334</v>
+        <v>49</v>
       </c>
       <c r="AM21" t="s">
         <v>72</v>
       </c>
       <c r="AN21" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
       <c r="AO21" t="s">
-        <v>335</v>
+        <v>49</v>
       </c>
       <c r="AP21" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" t="s">
-        <v>337</v>
-      </c>
-      <c r="D22" t="s">
-        <v>338</v>
-      </c>
-      <c r="E22" t="s">
         <v>339</v>
-      </c>
-      <c r="F22" t="s">
-        <v>340</v>
-      </c>
-      <c r="G22" t="s">
-        <v>341</v>
-      </c>
-      <c r="H22" t="s">
-        <v>49</v>
-      </c>
-      <c r="I22" t="s">
-        <v>342</v>
-      </c>
-      <c r="J22" t="s">
-        <v>343</v>
-      </c>
-      <c r="K22" t="s">
-        <v>318</v>
-      </c>
-      <c r="L22" t="s">
-        <v>344</v>
-      </c>
-      <c r="M22" t="s">
-        <v>86</v>
-      </c>
-      <c r="N22" t="s">
-        <v>55</v>
-      </c>
-      <c r="O22" t="s">
-        <v>153</v>
-      </c>
-      <c r="P22" t="s">
-        <v>345</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>320</v>
-      </c>
-      <c r="R22" t="s">
-        <v>90</v>
-      </c>
-      <c r="S22" t="s">
-        <v>91</v>
-      </c>
-      <c r="T22" t="s">
-        <v>92</v>
-      </c>
-      <c r="U22" t="s">
-        <v>60</v>
-      </c>
-      <c r="V22" t="s">
-        <v>60</v>
-      </c>
-      <c r="W22" t="s">
-        <v>346</v>
-      </c>
-      <c r="X22" t="s">
-        <v>170</v>
-      </c>
-      <c r="Y22" t="s">
-        <v>344</v>
-      </c>
-      <c r="Z22" t="s">
-        <v>347</v>
-      </c>
-      <c r="AA22" t="s">
-        <v>348</v>
-      </c>
-      <c r="AB22" t="s">
-        <v>349</v>
-      </c>
-      <c r="AC22" t="s">
-        <v>185</v>
-      </c>
-      <c r="AD22" t="s">
-        <v>98</v>
-      </c>
-      <c r="AE22" t="s">
-        <v>86</v>
-      </c>
-      <c r="AF22" t="s">
-        <v>70</v>
-      </c>
-      <c r="AG22" t="s">
-        <v>70</v>
-      </c>
-      <c r="AH22" t="s">
-        <v>70</v>
-      </c>
-      <c r="AI22" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ22" t="s">
-        <v>70</v>
-      </c>
-      <c r="AK22" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL22" t="s">
-        <v>49</v>
-      </c>
-      <c r="AM22" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN22" t="s">
-        <v>49</v>
-      </c>
-      <c r="AO22" t="s">
-        <v>49</v>
-      </c>
-      <c r="AP22" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" t="s">
-        <v>351</v>
-      </c>
-      <c r="D23" t="s">
-        <v>352</v>
-      </c>
-      <c r="E23" t="s">
-        <v>353</v>
-      </c>
-      <c r="F23" t="s">
-        <v>47</v>
-      </c>
-      <c r="G23" t="s">
-        <v>354</v>
-      </c>
-      <c r="H23" t="s">
-        <v>355</v>
-      </c>
-      <c r="I23" t="s">
-        <v>356</v>
-      </c>
-      <c r="J23" t="s">
-        <v>357</v>
-      </c>
-      <c r="K23" t="s">
-        <v>319</v>
-      </c>
-      <c r="L23" t="s">
-        <v>319</v>
-      </c>
-      <c r="M23" t="s">
-        <v>86</v>
-      </c>
-      <c r="N23" t="s">
-        <v>55</v>
-      </c>
-      <c r="O23" t="s">
-        <v>153</v>
-      </c>
-      <c r="P23" t="s">
-        <v>345</v>
-      </c>
-      <c r="Q23" t="s">
-        <v>320</v>
-      </c>
-      <c r="R23" t="s">
-        <v>90</v>
-      </c>
-      <c r="S23" t="s">
-        <v>91</v>
-      </c>
-      <c r="T23" t="s">
-        <v>92</v>
-      </c>
-      <c r="U23" t="s">
-        <v>60</v>
-      </c>
-      <c r="V23" t="s">
-        <v>60</v>
-      </c>
-      <c r="W23" t="s">
-        <v>93</v>
-      </c>
-      <c r="X23" t="s">
-        <v>94</v>
-      </c>
-      <c r="Y23" t="s">
-        <v>319</v>
-      </c>
-      <c r="Z23" t="s">
-        <v>95</v>
-      </c>
-      <c r="AA23" t="s">
-        <v>358</v>
-      </c>
-      <c r="AB23" t="s">
-        <v>321</v>
-      </c>
-      <c r="AC23" t="s">
-        <v>185</v>
-      </c>
-      <c r="AD23" t="s">
-        <v>98</v>
-      </c>
-      <c r="AE23" t="s">
-        <v>86</v>
-      </c>
-      <c r="AF23" t="s">
-        <v>70</v>
-      </c>
-      <c r="AG23" t="s">
-        <v>70</v>
-      </c>
-      <c r="AH23" t="s">
-        <v>70</v>
-      </c>
-      <c r="AI23" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ23" t="s">
-        <v>70</v>
-      </c>
-      <c r="AK23" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL23" t="s">
-        <v>49</v>
-      </c>
-      <c r="AM23" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN23" t="s">
-        <v>49</v>
-      </c>
-      <c r="AO23" t="s">
-        <v>49</v>
-      </c>
-      <c r="AP23" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" t="s">
-        <v>360</v>
-      </c>
-      <c r="D24" t="s">
-        <v>361</v>
-      </c>
-      <c r="E24" t="s">
-        <v>362</v>
-      </c>
-      <c r="F24" t="s">
-        <v>47</v>
-      </c>
-      <c r="G24" t="s">
-        <v>363</v>
-      </c>
-      <c r="H24" t="s">
-        <v>364</v>
-      </c>
-      <c r="I24" t="s">
-        <v>365</v>
-      </c>
-      <c r="J24" t="s">
-        <v>366</v>
-      </c>
-      <c r="K24" t="s">
-        <v>344</v>
-      </c>
-      <c r="L24" t="s">
-        <v>344</v>
-      </c>
-      <c r="M24" t="s">
-        <v>54</v>
-      </c>
-      <c r="N24" t="s">
-        <v>55</v>
-      </c>
-      <c r="O24" t="s">
-        <v>49</v>
-      </c>
-      <c r="P24" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>198</v>
-      </c>
-      <c r="R24" t="s">
-        <v>209</v>
-      </c>
-      <c r="S24" t="s">
-        <v>209</v>
-      </c>
-      <c r="T24" t="s">
-        <v>209</v>
-      </c>
-      <c r="U24" t="s">
-        <v>60</v>
-      </c>
-      <c r="V24" t="s">
-        <v>60</v>
-      </c>
-      <c r="W24" t="s">
-        <v>367</v>
-      </c>
-      <c r="X24" t="s">
-        <v>347</v>
-      </c>
-      <c r="Y24" t="s">
-        <v>344</v>
-      </c>
-      <c r="Z24" t="s">
-        <v>368</v>
-      </c>
-      <c r="AA24" t="s">
-        <v>199</v>
-      </c>
-      <c r="AB24" t="s">
-        <v>369</v>
-      </c>
-      <c r="AC24" t="s">
-        <v>185</v>
-      </c>
-      <c r="AD24" t="s">
-        <v>68</v>
-      </c>
-      <c r="AE24" t="s">
-        <v>69</v>
-      </c>
-      <c r="AF24" t="s">
-        <v>70</v>
-      </c>
-      <c r="AG24" t="s">
-        <v>70</v>
-      </c>
-      <c r="AH24" t="s">
-        <v>70</v>
-      </c>
-      <c r="AI24" t="s">
-        <v>49</v>
-      </c>
-      <c r="AJ24" t="s">
-        <v>70</v>
-      </c>
-      <c r="AK24" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL24" t="s">
-        <v>71</v>
-      </c>
-      <c r="AM24" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN24" t="s">
-        <v>370</v>
-      </c>
-      <c r="AO24" t="s">
-        <v>371</v>
-      </c>
-      <c r="AP24" t="s">
-        <v>372</v>
       </c>
     </row>
   </sheetData>

</xml_diff>